<commit_message>
RA workbook: recut against the finished dashboard, and stop typing the column names
The workbook was generated before s68 and s69 were rebuilt, so it was
already describing a screen that no longer existed.

It also kept its OWN copy of the column names, and they had drifted: it
said 'requestors (departments and RMs)' where s69 and the screen both
say '(departments / RMs)', and it dropped the '(year, month)' qualifier
the client puts on ten of the fourteen columns. That is the exact fault
the contents workbook is generated to avoid, so the extractor now reads
the column names, the summary bands and the open asks off the rendered
DOM and the builder holds no second copy of any of them.

Both workbooks regenerated. Every location column totals the client's
own published s67 figure, checked by live formula in the workbook and
by assert in the page.
</commit_message>
<xml_diff>
--- a/EDRMS_RA_Gap_Checker_2026-08-24.xlsx
+++ b/EDRMS_RA_Gap_Checker_2026-08-24.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Records and Archive Holdings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Records and Archive Holdings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Records and Archive Holdings'!$A$4:$H$51</definedName>

</xml_diff>